<commit_message>
atualiza logica e altera planilha de clientes
</commit_message>
<xml_diff>
--- a/followup-consultivo-trabalhista.xlsx
+++ b/followup-consultivo-trabalhista.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8E76806-DD68-4A15-BF75-72AA2B85F51A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4424AD4-16E2-42DE-90DD-81C9B0576B21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5640" yWindow="3855" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Configuração" sheetId="3" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="158">
   <si>
     <t>Cliente</t>
   </si>
@@ -325,6 +325,180 @@
   </si>
   <si>
     <t>karin.gambaro@dartibalefaria.com;moisesmiguel.garcia@dartibalefaria.com</t>
+  </si>
+  <si>
+    <t>Bsafer</t>
+  </si>
+  <si>
+    <t>06ed98c8-15f2-4048-b8c8-7440626c6697</t>
+  </si>
+  <si>
+    <t>Seguro Mary Help</t>
+  </si>
+  <si>
+    <t>977696f5-c896-469f-9b7e-40c4f9f4b01c</t>
+  </si>
+  <si>
+    <t>Urban Clinique</t>
+  </si>
+  <si>
+    <t>e8cee203-c77c-4108-a126-1ff6f4d3c092</t>
+  </si>
+  <si>
+    <t>Grupo Mary Help</t>
+  </si>
+  <si>
+    <t>bf4bfcac-4298-447d-ac35-dc777fcf7b58</t>
+  </si>
+  <si>
+    <t>Grupo Velox</t>
+  </si>
+  <si>
+    <t>395166f2-4f34-4ee1-872e-ec7dfa82ff8d</t>
+  </si>
+  <si>
+    <t>Black Madre</t>
+  </si>
+  <si>
+    <t>f812c45c-6690-4788-98a0-a63ccdd5c4d7</t>
+  </si>
+  <si>
+    <t>Grupo Banneg</t>
+  </si>
+  <si>
+    <t>1ff0478f-a874-4589-b556-c6da588f9b02</t>
+  </si>
+  <si>
+    <t>SmartCred</t>
+  </si>
+  <si>
+    <t>45b3b1d2-f785-4e97-aaeb-cc8968966e67</t>
+  </si>
+  <si>
+    <t>TFlow</t>
+  </si>
+  <si>
+    <t>5910fb59-5846-401f-b1e8-10e9cbf1e0d5</t>
+  </si>
+  <si>
+    <t>Cards Tecnologia</t>
+  </si>
+  <si>
+    <t>f7de8e8d-58d5-4bfa-8e16-8578a1b6b49b</t>
+  </si>
+  <si>
+    <t>Repitikos</t>
+  </si>
+  <si>
+    <t>29162db3-fb10-4638-b916-178044879e02</t>
+  </si>
+  <si>
+    <t>Espaço Católico São Bento</t>
+  </si>
+  <si>
+    <t>d17ac077-42fa-4707-915f-c315fdc6f609</t>
+  </si>
+  <si>
+    <t>Lav Me</t>
+  </si>
+  <si>
+    <t>cffbd86b-7ec4-44aa-8049-3cfe20586532</t>
+  </si>
+  <si>
+    <t>Talles Coelho Howard</t>
+  </si>
+  <si>
+    <t>01ef7328-2415-43d5-89c6-cd894de12a64</t>
+  </si>
+  <si>
+    <t>Sweet Futures Brazil</t>
+  </si>
+  <si>
+    <t>34c3a7c3-cfd5-44de-8699-5d248ffb539d</t>
+  </si>
+  <si>
+    <t>Ean Química Espu Mais</t>
+  </si>
+  <si>
+    <t>b973cd00-1c17-40c5-b5d7-561c61bab8e0</t>
+  </si>
+  <si>
+    <t>Laser Fast</t>
+  </si>
+  <si>
+    <t>fa3fea59-e88b-4758-bbb1-98ee30a4937b</t>
+  </si>
+  <si>
+    <t>Grupo NFT - Liberta Laser</t>
+  </si>
+  <si>
+    <t>8771ffb2-8621-4741-a028-33ddf246a193</t>
+  </si>
+  <si>
+    <t>IZI Estruturas</t>
+  </si>
+  <si>
+    <t>955ee7d6-ed46-4124-b94d-f8d404616527</t>
+  </si>
+  <si>
+    <t>Bless Lab</t>
+  </si>
+  <si>
+    <t>c322b442-3c55-4f69-8bd1-3768e53f29ca</t>
+  </si>
+  <si>
+    <t>Rafael Bertolucci</t>
+  </si>
+  <si>
+    <t>fb9dedf7-79a4-4daa-b69b-b8d4e142de02</t>
+  </si>
+  <si>
+    <t>Locação</t>
+  </si>
+  <si>
+    <t>ceae2d9c-36f6-4282-ad90-13a9e278b268</t>
+  </si>
+  <si>
+    <t>HM Pro</t>
+  </si>
+  <si>
+    <t>a889d91a-41b7-4fcd-9735-f12741c554a9</t>
+  </si>
+  <si>
+    <t>Megaspark</t>
+  </si>
+  <si>
+    <t>53d1196f-8fee-482a-a856-d818aeae8142</t>
+  </si>
+  <si>
+    <t>Bitflowin</t>
+  </si>
+  <si>
+    <t>e41e1cd8-e3f6-412a-a94f-919df7d83427</t>
+  </si>
+  <si>
+    <t>NewM</t>
+  </si>
+  <si>
+    <t>414fcda7-1be9-4060-ac90-bc0fca31a946</t>
+  </si>
+  <si>
+    <t>Desce Lava</t>
+  </si>
+  <si>
+    <t>a923182b-14ae-406a-937f-1a68927e2174</t>
+  </si>
+  <si>
+    <t>Cyan</t>
+  </si>
+  <si>
+    <t>cdce77a6-0591-4119-8bb0-d6f0db396e97</t>
+  </si>
+  <si>
+    <t>Cachorrão do Claudião</t>
+  </si>
+  <si>
+    <t>c8a9dc20-9d78-4775-9fe9-f8d5411c957a</t>
   </si>
 </sst>
 </file>
@@ -747,7 +921,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00FB8B67-ADAA-4E80-BCAD-03B366569374}">
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D77"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
@@ -1429,6 +1603,412 @@
         <v>97</v>
       </c>
     </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>100</v>
+      </c>
+      <c r="B49" t="s">
+        <v>101</v>
+      </c>
+      <c r="C49" t="s">
+        <v>99</v>
+      </c>
+      <c r="D49" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>102</v>
+      </c>
+      <c r="B50" t="s">
+        <v>103</v>
+      </c>
+      <c r="C50" t="s">
+        <v>99</v>
+      </c>
+      <c r="D50" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>104</v>
+      </c>
+      <c r="B51" t="s">
+        <v>105</v>
+      </c>
+      <c r="C51" t="s">
+        <v>99</v>
+      </c>
+      <c r="D51" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>106</v>
+      </c>
+      <c r="B52" t="s">
+        <v>107</v>
+      </c>
+      <c r="C52" t="s">
+        <v>99</v>
+      </c>
+      <c r="D52" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>108</v>
+      </c>
+      <c r="B53" t="s">
+        <v>109</v>
+      </c>
+      <c r="C53" t="s">
+        <v>99</v>
+      </c>
+      <c r="D53" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>110</v>
+      </c>
+      <c r="B54" t="s">
+        <v>111</v>
+      </c>
+      <c r="C54" t="s">
+        <v>99</v>
+      </c>
+      <c r="D54" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>112</v>
+      </c>
+      <c r="B55" t="s">
+        <v>113</v>
+      </c>
+      <c r="C55" t="s">
+        <v>99</v>
+      </c>
+      <c r="D55" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>114</v>
+      </c>
+      <c r="B56" t="s">
+        <v>115</v>
+      </c>
+      <c r="C56" t="s">
+        <v>99</v>
+      </c>
+      <c r="D56" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>116</v>
+      </c>
+      <c r="B57" t="s">
+        <v>117</v>
+      </c>
+      <c r="C57" t="s">
+        <v>99</v>
+      </c>
+      <c r="D57" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>118</v>
+      </c>
+      <c r="B58" t="s">
+        <v>119</v>
+      </c>
+      <c r="C58" t="s">
+        <v>99</v>
+      </c>
+      <c r="D58" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>120</v>
+      </c>
+      <c r="B59" t="s">
+        <v>121</v>
+      </c>
+      <c r="C59" t="s">
+        <v>99</v>
+      </c>
+      <c r="D59" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>122</v>
+      </c>
+      <c r="B60" t="s">
+        <v>123</v>
+      </c>
+      <c r="C60" t="s">
+        <v>99</v>
+      </c>
+      <c r="D60" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>124</v>
+      </c>
+      <c r="B61" t="s">
+        <v>125</v>
+      </c>
+      <c r="C61" t="s">
+        <v>99</v>
+      </c>
+      <c r="D61" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>126</v>
+      </c>
+      <c r="B62" t="s">
+        <v>127</v>
+      </c>
+      <c r="C62" t="s">
+        <v>99</v>
+      </c>
+      <c r="D62" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>128</v>
+      </c>
+      <c r="B63" t="s">
+        <v>129</v>
+      </c>
+      <c r="C63" t="s">
+        <v>99</v>
+      </c>
+      <c r="D63" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>130</v>
+      </c>
+      <c r="B64" t="s">
+        <v>131</v>
+      </c>
+      <c r="C64" t="s">
+        <v>99</v>
+      </c>
+      <c r="D64" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>132</v>
+      </c>
+      <c r="B65" t="s">
+        <v>133</v>
+      </c>
+      <c r="C65" t="s">
+        <v>99</v>
+      </c>
+      <c r="D65" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>134</v>
+      </c>
+      <c r="B66" t="s">
+        <v>135</v>
+      </c>
+      <c r="C66" t="s">
+        <v>99</v>
+      </c>
+      <c r="D66" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>136</v>
+      </c>
+      <c r="B67" t="s">
+        <v>137</v>
+      </c>
+      <c r="C67" t="s">
+        <v>99</v>
+      </c>
+      <c r="D67" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>138</v>
+      </c>
+      <c r="B68" t="s">
+        <v>139</v>
+      </c>
+      <c r="C68" t="s">
+        <v>99</v>
+      </c>
+      <c r="D68" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>140</v>
+      </c>
+      <c r="B69" t="s">
+        <v>141</v>
+      </c>
+      <c r="C69" t="s">
+        <v>99</v>
+      </c>
+      <c r="D69" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>142</v>
+      </c>
+      <c r="B70" t="s">
+        <v>143</v>
+      </c>
+      <c r="C70" t="s">
+        <v>99</v>
+      </c>
+      <c r="D70" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>144</v>
+      </c>
+      <c r="B71" t="s">
+        <v>145</v>
+      </c>
+      <c r="C71" t="s">
+        <v>99</v>
+      </c>
+      <c r="D71" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>146</v>
+      </c>
+      <c r="B72" t="s">
+        <v>147</v>
+      </c>
+      <c r="C72" t="s">
+        <v>99</v>
+      </c>
+      <c r="D72" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>148</v>
+      </c>
+      <c r="B73" t="s">
+        <v>149</v>
+      </c>
+      <c r="C73" t="s">
+        <v>99</v>
+      </c>
+      <c r="D73" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>150</v>
+      </c>
+      <c r="B74" t="s">
+        <v>151</v>
+      </c>
+      <c r="C74" t="s">
+        <v>99</v>
+      </c>
+      <c r="D74" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>152</v>
+      </c>
+      <c r="B75" t="s">
+        <v>153</v>
+      </c>
+      <c r="C75" t="s">
+        <v>99</v>
+      </c>
+      <c r="D75" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>154</v>
+      </c>
+      <c r="B76" t="s">
+        <v>155</v>
+      </c>
+      <c r="C76" t="s">
+        <v>99</v>
+      </c>
+      <c r="D76" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>156</v>
+      </c>
+      <c r="B77" t="s">
+        <v>157</v>
+      </c>
+      <c r="C77" t="s">
+        <v>99</v>
+      </c>
+      <c r="D77" t="s">
+        <v>157</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>